<commit_message>
fix: fixes vocabulary mapping
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-dataservice.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-dataservice.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-14 10:30:30</t>
+          <t>2026-10-14 14:14:49</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1727,7 +1727,11 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>( &lt;http://publications.europa.eu/resource/authority/access-right/PUBLIC&gt; &lt;http://publications.europa.eu/resource/authority/access-right/RESTRICTED&gt; &lt;http://publications.europa.eu/resource/authority/access-right/NON_PUBLIC&gt; )</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -1739,7 +1743,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>dash:URIEditor</t>
+          <t>dash:EnumSelectEditor</t>
         </is>
       </c>
     </row>

</xml_diff>